<commit_message>
Add crew avatars, videos, and fix RPC for all 19 crews
- Add 12 new avatar photos and 6 new crew videos
- Fix 7 placeholder crews (rename Экипаж N to real names)
- Fix RPC get_crews_full: correct metric names (distribution/contracts/liga_pro/contacts) and add totalScore/finishTarget
- Fix Track.tsx: guard against NaN in getPointAtLength
- Add video error fallback and loop in TeamDetail
- Add video_url field to CrewForm

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Admin/Admin.xlsx
+++ b/Admin/Admin.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruslan\Desktop\Нейросети\Projects\forsazh\Admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD732F7A-7EB7-4944-A992-1FC14D19B329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EED513-D029-42DB-971D-8FD3B2A93735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FC3B7296-589A-4A51-93A7-BEFBADEFDE12}"/>
   </bookViews>
   <sheets>
     <sheet name="Экипажи" sheetId="3" r:id="rId1"/>
-    <sheet name="Экипажи награды Март" sheetId="2" r:id="rId2"/>
-    <sheet name="Трасса" sheetId="4" r:id="rId3"/>
-    <sheet name="Награды" sheetId="1" r:id="rId4"/>
+    <sheet name="Экипажи по месяцам" sheetId="5" r:id="rId2"/>
+    <sheet name="Экипажи награды Март" sheetId="2" r:id="rId3"/>
+    <sheet name="Трасса" sheetId="4" r:id="rId4"/>
+    <sheet name="Награды" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="136">
   <si>
     <t>#1 по контрактованию</t>
   </si>
@@ -388,6 +389,63 @@
   </si>
   <si>
     <t>Финишь</t>
+  </si>
+  <si>
+    <t>Крымская весна</t>
+  </si>
+  <si>
+    <t>Дальневосточный гром</t>
+  </si>
+  <si>
+    <t>Амурский тигр</t>
+  </si>
+  <si>
+    <t>Ледовый шторм</t>
+  </si>
+  <si>
+    <t>Байкальский лёд</t>
+  </si>
+  <si>
+    <t>Морской бриз</t>
+  </si>
+  <si>
+    <t>Хакасский беркут</t>
+  </si>
+  <si>
+    <t>Русский остров</t>
+  </si>
+  <si>
+    <t>Армавирский сокол</t>
+  </si>
+  <si>
+    <t>Морской бастион</t>
+  </si>
+  <si>
+    <t>Казачий острог</t>
+  </si>
+  <si>
+    <t>Приморский дракон</t>
+  </si>
+  <si>
+    <t>Ворошиловская батарея</t>
+  </si>
+  <si>
+    <t>Енисейский порог</t>
+  </si>
+  <si>
+    <t>Кубанская застава</t>
+  </si>
+  <si>
+    <t>Армавирский щит</t>
+  </si>
+  <si>
+    <t>Кремлёвский утёс</t>
+  </si>
+  <si>
+    <t>Спасская башня</t>
+  </si>
+  <si>
+    <t>Царицынский бастион</t>
   </si>
 </sst>
 </file>
@@ -475,7 +533,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -755,12 +813,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -836,6 +914,46 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -845,7 +963,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1164,7 +1281,7 @@
   <dimension ref="A1:M29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="4" max="4" width="23.5703125" customWidth="1"/>
@@ -1209,8 +1326,8 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>22</v>
+      <c r="A2" s="4" t="s">
+        <v>133</v>
       </c>
       <c r="B2" t="s">
         <v>44</v>
@@ -1242,8 +1359,8 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>23</v>
+      <c r="A3" s="4" t="s">
+        <v>134</v>
       </c>
       <c r="B3" t="s">
         <v>46</v>
@@ -1279,8 +1396,8 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>24</v>
+      <c r="A4" s="4" t="s">
+        <v>135</v>
       </c>
       <c r="B4" t="s">
         <v>48</v>
@@ -1316,8 +1433,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>25</v>
+      <c r="A5" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="B5" t="s">
         <v>49</v>
@@ -1353,8 +1470,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>26</v>
+      <c r="A6" s="4" t="s">
+        <v>131</v>
       </c>
       <c r="B6" t="s">
         <v>49</v>
@@ -1390,8 +1507,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>27</v>
+      <c r="A7" s="4" t="s">
+        <v>132</v>
       </c>
       <c r="B7" t="s">
         <v>50</v>
@@ -1427,8 +1544,8 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>28</v>
+      <c r="A8" s="4" t="s">
+        <v>125</v>
       </c>
       <c r="B8" t="s">
         <v>50</v>
@@ -1464,8 +1581,8 @@
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
+      <c r="A9" s="4" t="s">
+        <v>122</v>
       </c>
       <c r="B9" t="s">
         <v>52</v>
@@ -1501,8 +1618,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>30</v>
+      <c r="A10" s="4" t="s">
+        <v>117</v>
       </c>
       <c r="B10" t="s">
         <v>52</v>
@@ -1539,8 +1656,8 @@
       <c r="M10" s="2"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>31</v>
+      <c r="A11" s="4" t="s">
+        <v>126</v>
       </c>
       <c r="B11" t="s">
         <v>52</v>
@@ -1576,8 +1693,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>32</v>
+      <c r="A12" s="4" t="s">
+        <v>123</v>
       </c>
       <c r="B12" t="s">
         <v>55</v>
@@ -1613,8 +1730,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>33</v>
+      <c r="A13" s="4" t="s">
+        <v>130</v>
       </c>
       <c r="B13" t="s">
         <v>55</v>
@@ -1650,8 +1767,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>34</v>
+      <c r="A14" s="4" t="s">
+        <v>128</v>
       </c>
       <c r="B14" t="s">
         <v>57</v>
@@ -1687,8 +1804,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>35</v>
+      <c r="A15" s="4" t="s">
+        <v>129</v>
       </c>
       <c r="B15" t="s">
         <v>57</v>
@@ -1724,8 +1841,8 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>36</v>
+      <c r="A16" s="4" t="s">
+        <v>124</v>
       </c>
       <c r="B16" t="s">
         <v>57</v>
@@ -1761,8 +1878,8 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>37</v>
+      <c r="A17" s="4" t="s">
+        <v>121</v>
       </c>
       <c r="B17" t="s">
         <v>59</v>
@@ -1798,8 +1915,8 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>38</v>
+      <c r="A18" s="4" t="s">
+        <v>120</v>
       </c>
       <c r="B18" t="s">
         <v>59</v>
@@ -1835,8 +1952,8 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>39</v>
+      <c r="A19" s="4" t="s">
+        <v>119</v>
       </c>
       <c r="B19" t="s">
         <v>60</v>
@@ -1871,9 +1988,9 @@
         <v>543</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>40</v>
+    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="B20" t="s">
         <v>60</v>
@@ -1920,6 +2037,969 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C254EAB-5EAB-4F09-9690-CAC87533A1C2}">
+  <dimension ref="A1:R30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="7" max="7" width="17.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" customWidth="1"/>
+    <col min="16" max="16" width="13.140625" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G1" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="F2" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="K2" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="M2" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="O2" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="P2" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q2" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="R2" s="25" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="47">
+        <f>SUM(G3:J3)</f>
+        <v>798</v>
+      </c>
+      <c r="G3" s="40">
+        <v>79</v>
+      </c>
+      <c r="H3" s="41">
+        <v>332</v>
+      </c>
+      <c r="I3" s="41">
+        <v>354</v>
+      </c>
+      <c r="J3" s="42">
+        <v>33</v>
+      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="6"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="47">
+        <f t="shared" ref="F4:F21" si="0">SUM(G4:J4)</f>
+        <v>918</v>
+      </c>
+      <c r="G4" s="40">
+        <v>109</v>
+      </c>
+      <c r="H4" s="41">
+        <f t="shared" ref="H4:J19" si="1">H3+30</f>
+        <v>362</v>
+      </c>
+      <c r="I4" s="41">
+        <f t="shared" si="1"/>
+        <v>384</v>
+      </c>
+      <c r="J4" s="42">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="6"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" s="47">
+        <f t="shared" si="0"/>
+        <v>1038</v>
+      </c>
+      <c r="G5" s="40">
+        <v>139</v>
+      </c>
+      <c r="H5" s="41">
+        <f t="shared" si="1"/>
+        <v>392</v>
+      </c>
+      <c r="I5" s="41">
+        <f t="shared" si="1"/>
+        <v>414</v>
+      </c>
+      <c r="J5" s="42">
+        <f t="shared" si="1"/>
+        <v>93</v>
+      </c>
+      <c r="K5" s="4"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="6"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="47">
+        <f t="shared" si="0"/>
+        <v>1158</v>
+      </c>
+      <c r="G6" s="40">
+        <v>169</v>
+      </c>
+      <c r="H6" s="41">
+        <f t="shared" si="1"/>
+        <v>422</v>
+      </c>
+      <c r="I6" s="41">
+        <f t="shared" si="1"/>
+        <v>444</v>
+      </c>
+      <c r="J6" s="42">
+        <f t="shared" si="1"/>
+        <v>123</v>
+      </c>
+      <c r="K6" s="4"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="6"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="47">
+        <f t="shared" si="0"/>
+        <v>1278</v>
+      </c>
+      <c r="G7" s="40">
+        <v>199</v>
+      </c>
+      <c r="H7" s="41">
+        <f t="shared" si="1"/>
+        <v>452</v>
+      </c>
+      <c r="I7" s="41">
+        <f t="shared" si="1"/>
+        <v>474</v>
+      </c>
+      <c r="J7" s="42">
+        <f t="shared" si="1"/>
+        <v>153</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="6"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" s="47">
+        <f t="shared" si="0"/>
+        <v>1398</v>
+      </c>
+      <c r="G8" s="40">
+        <v>229</v>
+      </c>
+      <c r="H8" s="41">
+        <f t="shared" si="1"/>
+        <v>482</v>
+      </c>
+      <c r="I8" s="41">
+        <f t="shared" si="1"/>
+        <v>504</v>
+      </c>
+      <c r="J8" s="42">
+        <f t="shared" si="1"/>
+        <v>183</v>
+      </c>
+      <c r="K8" s="4"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="6"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="47">
+        <f t="shared" si="0"/>
+        <v>1518</v>
+      </c>
+      <c r="G9" s="40">
+        <v>259</v>
+      </c>
+      <c r="H9" s="41">
+        <f t="shared" si="1"/>
+        <v>512</v>
+      </c>
+      <c r="I9" s="41">
+        <f t="shared" si="1"/>
+        <v>534</v>
+      </c>
+      <c r="J9" s="42">
+        <f t="shared" si="1"/>
+        <v>213</v>
+      </c>
+      <c r="K9" s="4"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="6"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="47">
+        <f t="shared" si="0"/>
+        <v>1638</v>
+      </c>
+      <c r="G10" s="40">
+        <v>289</v>
+      </c>
+      <c r="H10" s="41">
+        <f t="shared" si="1"/>
+        <v>542</v>
+      </c>
+      <c r="I10" s="41">
+        <f t="shared" si="1"/>
+        <v>564</v>
+      </c>
+      <c r="J10" s="42">
+        <f t="shared" si="1"/>
+        <v>243</v>
+      </c>
+      <c r="K10" s="4"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="6"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" s="47">
+        <f t="shared" si="0"/>
+        <v>1758</v>
+      </c>
+      <c r="G11" s="40">
+        <v>319</v>
+      </c>
+      <c r="H11" s="41">
+        <f t="shared" si="1"/>
+        <v>572</v>
+      </c>
+      <c r="I11" s="41">
+        <f t="shared" si="1"/>
+        <v>594</v>
+      </c>
+      <c r="J11" s="42">
+        <f t="shared" si="1"/>
+        <v>273</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="6"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="47">
+        <f t="shared" si="0"/>
+        <v>1878</v>
+      </c>
+      <c r="G12" s="40">
+        <v>349</v>
+      </c>
+      <c r="H12" s="41">
+        <f t="shared" si="1"/>
+        <v>602</v>
+      </c>
+      <c r="I12" s="41">
+        <f t="shared" si="1"/>
+        <v>624</v>
+      </c>
+      <c r="J12" s="42">
+        <f t="shared" si="1"/>
+        <v>303</v>
+      </c>
+      <c r="K12" s="4"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="6"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F13" s="47">
+        <f t="shared" si="0"/>
+        <v>1998</v>
+      </c>
+      <c r="G13" s="40">
+        <v>379</v>
+      </c>
+      <c r="H13" s="41">
+        <f t="shared" si="1"/>
+        <v>632</v>
+      </c>
+      <c r="I13" s="41">
+        <f t="shared" si="1"/>
+        <v>654</v>
+      </c>
+      <c r="J13" s="42">
+        <f t="shared" si="1"/>
+        <v>333</v>
+      </c>
+      <c r="K13" s="4"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="6"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F14" s="47">
+        <f t="shared" si="0"/>
+        <v>2118</v>
+      </c>
+      <c r="G14" s="40">
+        <v>409</v>
+      </c>
+      <c r="H14" s="41">
+        <f t="shared" si="1"/>
+        <v>662</v>
+      </c>
+      <c r="I14" s="41">
+        <f t="shared" si="1"/>
+        <v>684</v>
+      </c>
+      <c r="J14" s="42">
+        <f t="shared" si="1"/>
+        <v>363</v>
+      </c>
+      <c r="K14" s="4"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="6"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="47">
+        <f t="shared" si="0"/>
+        <v>2238</v>
+      </c>
+      <c r="G15" s="40">
+        <v>439</v>
+      </c>
+      <c r="H15" s="41">
+        <f t="shared" si="1"/>
+        <v>692</v>
+      </c>
+      <c r="I15" s="41">
+        <f t="shared" si="1"/>
+        <v>714</v>
+      </c>
+      <c r="J15" s="42">
+        <f t="shared" si="1"/>
+        <v>393</v>
+      </c>
+      <c r="K15" s="4"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="6"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" s="47">
+        <f t="shared" si="0"/>
+        <v>2358</v>
+      </c>
+      <c r="G16" s="40">
+        <v>469</v>
+      </c>
+      <c r="H16" s="41">
+        <f t="shared" si="1"/>
+        <v>722</v>
+      </c>
+      <c r="I16" s="41">
+        <f t="shared" si="1"/>
+        <v>744</v>
+      </c>
+      <c r="J16" s="42">
+        <f t="shared" si="1"/>
+        <v>423</v>
+      </c>
+      <c r="K16" s="4"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="6"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="F17" s="47">
+        <f t="shared" si="0"/>
+        <v>2478</v>
+      </c>
+      <c r="G17" s="40">
+        <v>499</v>
+      </c>
+      <c r="H17" s="41">
+        <f t="shared" si="1"/>
+        <v>752</v>
+      </c>
+      <c r="I17" s="41">
+        <f t="shared" si="1"/>
+        <v>774</v>
+      </c>
+      <c r="J17" s="42">
+        <f t="shared" si="1"/>
+        <v>453</v>
+      </c>
+      <c r="K17" s="4"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="6"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="47">
+        <f t="shared" si="0"/>
+        <v>2598</v>
+      </c>
+      <c r="G18" s="40">
+        <v>529</v>
+      </c>
+      <c r="H18" s="41">
+        <f t="shared" si="1"/>
+        <v>782</v>
+      </c>
+      <c r="I18" s="41">
+        <f t="shared" si="1"/>
+        <v>804</v>
+      </c>
+      <c r="J18" s="42">
+        <f t="shared" si="1"/>
+        <v>483</v>
+      </c>
+      <c r="K18" s="4"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="6"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" s="47">
+        <f t="shared" si="0"/>
+        <v>2718</v>
+      </c>
+      <c r="G19" s="40">
+        <v>559</v>
+      </c>
+      <c r="H19" s="41">
+        <f t="shared" si="1"/>
+        <v>812</v>
+      </c>
+      <c r="I19" s="41">
+        <f t="shared" si="1"/>
+        <v>834</v>
+      </c>
+      <c r="J19" s="42">
+        <f t="shared" si="1"/>
+        <v>513</v>
+      </c>
+      <c r="K19" s="4"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="6"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F20" s="47">
+        <f t="shared" si="0"/>
+        <v>2838</v>
+      </c>
+      <c r="G20" s="40">
+        <v>589</v>
+      </c>
+      <c r="H20" s="41">
+        <f t="shared" ref="H20:J20" si="2">H19+30</f>
+        <v>842</v>
+      </c>
+      <c r="I20" s="41">
+        <f t="shared" si="2"/>
+        <v>864</v>
+      </c>
+      <c r="J20" s="42">
+        <f t="shared" si="2"/>
+        <v>543</v>
+      </c>
+      <c r="K20" s="4"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="6"/>
+    </row>
+    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="48">
+        <f t="shared" si="0"/>
+        <v>2958</v>
+      </c>
+      <c r="G21" s="43">
+        <v>619</v>
+      </c>
+      <c r="H21" s="44">
+        <f t="shared" ref="H21:J21" si="3">H20+30</f>
+        <v>872</v>
+      </c>
+      <c r="I21" s="44">
+        <f t="shared" si="3"/>
+        <v>894</v>
+      </c>
+      <c r="J21" s="45">
+        <f t="shared" si="3"/>
+        <v>573</v>
+      </c>
+      <c r="K21" s="7"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="9"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97A47090-AFD5-44B1-8B45-E3B64166D6ED}">
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1931,15 +3011,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="35"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="51"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -2159,7 +3239,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94158793-3403-4696-9063-65D735965823}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2282,7 +3362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{116A30D3-EEA8-4C91-9AA2-31961970EC9B}">
   <dimension ref="A2:C21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>